<commit_message>
[ROS-PS-v4.1.0] Correct form version metadata
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ROS-PS/v4.1.0/Form-ROS-PS-v4.1.0.xlsx
+++ b/form_reporting_templates/ROS-PS/v4.1.0/Form-ROS-PS-v4.1.0.xlsx
@@ -1614,8 +1614,10 @@
       <c r="F4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="11">
-        <v>4</v>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>4.1.0</t>
+        </is>
       </c>
       <c r="H4" s="12"/>
     </row>

</xml_diff>

<commit_message>
[ROS-PS-v4.1.0] Correct catalogue links
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ROS-PS/v4.1.0/Form-ROS-PS-v4.1.0.xlsx
+++ b/form_reporting_templates/ROS-PS/v4.1.0/Form-ROS-PS-v4.1.0.xlsx
@@ -6844,17 +6844,17 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E1" r:id="rId1" location="samplingMethodsForSamplingCollection" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
+    <hyperlink ref="E1" r:id="rId1" location="samplingMethodsForSamplingCollections" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
     <hyperlink ref="Q1" r:id="rId2" location="sex" xr:uid="{00000000-0004-0000-0900-000001000000}"/>
-    <hyperlink ref="F2" r:id="rId3" location="lengthMeasurementTypes" xr:uid="{00000000-0004-0000-0900-000002000000}"/>
+    <hyperlink ref="F2" r:id="rId3" location="allMeasurements" xr:uid="{00000000-0004-0000-0900-000002000000}"/>
     <hyperlink ref="H2" r:id="rId4" location="lengthMeasurementTools" xr:uid="{00000000-0004-0000-0900-000003000000}"/>
-    <hyperlink ref="J2" r:id="rId5" location="lengthMeasurementTypes" xr:uid="{00000000-0004-0000-0900-000004000000}"/>
+    <hyperlink ref="J2" r:id="rId5" location="allMeasurements" xr:uid="{00000000-0004-0000-0900-000004000000}"/>
     <hyperlink ref="L2" r:id="rId6" location="lengthMeasurementTools" xr:uid="{00000000-0004-0000-0900-000005000000}"/>
     <hyperlink ref="N2" r:id="rId7" location="fishProcessingTypes" xr:uid="{00000000-0004-0000-0900-000006000000}"/>
     <hyperlink ref="P2" r:id="rId8" location="weightMeasurementTools" xr:uid="{00000000-0004-0000-0900-000007000000}"/>
-    <hyperlink ref="S2" r:id="rId9" location="Maturity_Stages" xr:uid="{00000000-0004-0000-0900-000008000000}"/>
-    <hyperlink ref="T2" r:id="rId10" location="samplingMethodsForSamplingCollection" xr:uid="{00000000-0004-0000-0900-000009000000}"/>
-    <hyperlink ref="U2" r:id="rId11" location="fishStorageTypes" xr:uid="{00000000-0004-0000-0900-00000A000000}"/>
+    <hyperlink ref="S2" r:id="rId9" location="maturityStages" xr:uid="{00000000-0004-0000-0900-000008000000}"/>
+    <hyperlink ref="T2" r:id="rId10" location="biologicalMaterials" xr:uid="{00000000-0004-0000-0900-000009000000}"/>
+    <hyperlink ref="U2" r:id="rId11" location="samplePreservationMethods" xr:uid="{00000000-0004-0000-0900-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19488,9 +19488,9 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" location="countries" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="E4" r:id="rId2" location="Ports" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="E4" r:id="rId2" location="ports" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
     <hyperlink ref="I4" r:id="rId3" location="countries" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="J4" r:id="rId4" location="Ports" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="J4" r:id="rId4" location="ports" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
     <hyperlink ref="U4" r:id="rId5" location="reasonsDaysLost" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
     <hyperlink ref="V4" r:id="rId6" location="reasonsDaysLost" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
     <hyperlink ref="W4" r:id="rId7" location="reasonsDaysLost" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
@@ -23253,7 +23253,7 @@
     <hyperlink ref="K1" r:id="rId2" location="gears" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
     <hyperlink ref="C2" r:id="rId3" location="countries" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
     <hyperlink ref="G2" r:id="rId4" location="countries" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
-    <hyperlink ref="H2" r:id="rId5" location="Ports" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="H2" r:id="rId5" location="ports" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
     <hyperlink ref="M3" r:id="rId6" location="countries" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
     <hyperlink ref="O3" r:id="rId7" location="countries" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
   </hyperlinks>
@@ -25969,9 +25969,9 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" location="countries" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="C3" r:id="rId2" location="Ports" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="C3" r:id="rId2" location="ports" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
     <hyperlink ref="G3" r:id="rId3" location="countries" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
-    <hyperlink ref="H3" r:id="rId4" location="Ports" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
+    <hyperlink ref="H3" r:id="rId4" location="ports" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -34907,13 +34907,13 @@
     <hyperlink ref="P3" r:id="rId6" location="fishStorageTypes" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
     <hyperlink ref="Q3" r:id="rId7" location="fishStorageTypes" display="TYPE_2_CODE" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
     <hyperlink ref="R3" r:id="rId8" location="fishStorageTypes" display="TYPE_3_CODE" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
-    <hyperlink ref="AH3" r:id="rId9" location="wasteManagementCategories" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="AH3" r:id="rId9" location="wasteCategories" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
     <hyperlink ref="AI3" r:id="rId10" location="wasteDisposalMethods" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
-    <hyperlink ref="AJ3" r:id="rId11" location="wasteManagementCategories" display="CATEGORY_2_CODE" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
+    <hyperlink ref="AJ3" r:id="rId11" location="wasteCategories" display="CATEGORY_2_CODE" xr:uid="{00000000-0004-0000-0400-00000A000000}"/>
     <hyperlink ref="AK3" r:id="rId12" location="wasteDisposalMethods" display="STORAGE_DISPOSAL_METHOD_2_CODE" xr:uid="{00000000-0004-0000-0400-00000B000000}"/>
-    <hyperlink ref="AL3" r:id="rId13" location="wasteManagementCategories" display="CATEGORY_3_CODE" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
+    <hyperlink ref="AL3" r:id="rId13" location="wasteCategories" display="CATEGORY_3_CODE" xr:uid="{00000000-0004-0000-0400-00000C000000}"/>
     <hyperlink ref="AM3" r:id="rId14" location="wasteDisposalMethods" display="STORAGE_DISPOSAL_METHOD_3_CODE" xr:uid="{00000000-0004-0000-0400-00000D000000}"/>
-    <hyperlink ref="AN3" r:id="rId15" location="wasteManagementCategories" display="CATEGORY_4_CODE" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
+    <hyperlink ref="AN3" r:id="rId15" location="wasteCategories" display="CATEGORY_4_CODE" xr:uid="{00000000-0004-0000-0400-00000E000000}"/>
     <hyperlink ref="AO3" r:id="rId16" location="wasteDisposalMethods" display="STORAGE_DISPOSAL_METHOD_4_CODE" xr:uid="{00000000-0004-0000-0400-00000F000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -42842,8 +42842,8 @@
     <hyperlink ref="G3" r:id="rId4" location="schoolSightingCues" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
     <hyperlink ref="H3" r:id="rId5" location="schoolSightingCues" xr:uid="{00000000-0004-0000-0600-000004000000}"/>
     <hyperlink ref="I3" r:id="rId6" location="schoolSightingCues" xr:uid="{00000000-0004-0000-0600-000005000000}"/>
-    <hyperlink ref="U3" r:id="rId7" location="FADraftDesigns" xr:uid="{00000000-0004-0000-0600-000006000000}"/>
-    <hyperlink ref="V3" r:id="rId8" location="FADtailDesigns" xr:uid="{00000000-0004-0000-0600-000007000000}"/>
+    <hyperlink ref="U3" r:id="rId7" location="fadRaftDesigns" xr:uid="{00000000-0004-0000-0600-000006000000}"/>
+    <hyperlink ref="V3" r:id="rId8" location="fadTailDesigns" xr:uid="{00000000-0004-0000-0600-000007000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -44493,7 +44493,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D1" r:id="rId1" location="cetaceansAndWhaleSharks" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
+    <hyperlink ref="D1" r:id="rId1" location="cetaceanSpecies" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -47191,10 +47191,10 @@
   <hyperlinks>
     <hyperlink ref="D1" r:id="rId1" location="allSpecies" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
     <hyperlink ref="G1" r:id="rId2" location="samplingMethodsForCatchEstimation" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
-    <hyperlink ref="E2" r:id="rId3" location="typesOfFate" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
+    <hyperlink ref="E2" r:id="rId3" location="fateTypes" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
     <hyperlink ref="F2" r:id="rId4" location="fates" xr:uid="{00000000-0004-0000-0800-000003000000}"/>
     <hyperlink ref="I2" r:id="rId5" location="fishProcessingTypes" xr:uid="{00000000-0004-0000-0800-000004000000}"/>
-    <hyperlink ref="K2" r:id="rId6" location="weightEstimationMethods" xr:uid="{00000000-0004-0000-0800-000005000000}"/>
+    <hyperlink ref="K2" r:id="rId6" location="weightMeasurementTools" xr:uid="{00000000-0004-0000-0800-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>